<commit_message>
W02/D5: decision tool labels aligned with their wrapped text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01123CnpKxdZ7Th4XwviT5bS
</commit_message>
<xml_diff>
--- a/content/W02/D5/demos/C2_W02_D05_decision_tool_STUDENT.xlsx
+++ b/content/W02/D5/demos/C2_W02_D05_decision_tool_STUDENT.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -120,11 +120,16 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -742,7 +747,7 @@
       <c r="B5" s="8" t="n">
         <v>12400</v>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Member id to find</t>
         </is>
@@ -1039,7 +1044,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>The foot: total revenue (Rs)</t>
         </is>
@@ -1228,7 +1233,7 @@
           <t>Change on the comparison</t>
         </is>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="13">
         <f>(B5-B6)/B5</f>
         <v/>
       </c>
@@ -1474,7 +1479,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Tabs fixed</t>
         </is>

</xml_diff>